<commit_message>
Add flask app and add more timeout and add serve framework for add chanel timeout
</commit_message>
<xml_diff>
--- a/Createur/New_File2.xlsx
+++ b/Createur/New_File2.xlsx
@@ -424,7 +424,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>O Aaron</t>
+          <t>Aaron</t>
         </is>
       </c>
     </row>
@@ -436,7 +436,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>khamelonei</t>
+          <t>senkt</t>
         </is>
       </c>
     </row>
@@ -448,7 +448,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>khamelonontas</t>
+          <t>Senkung</t>
         </is>
       </c>
     </row>
@@ -460,7 +460,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>na meiosei</t>
+          <t>zu senken</t>
         </is>
       </c>
     </row>
@@ -472,7 +472,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>egkataleipo</t>
+          <t>aufgeben</t>
         </is>
       </c>
     </row>
@@ -484,7 +484,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>egkataleipontas</t>
+          <t>aufgeben</t>
         </is>
       </c>
     </row>
@@ -496,7 +496,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>egkataleimmenos</t>
+          <t>verlassen</t>
         </is>
       </c>
     </row>
@@ -508,7 +508,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>egkataleimmenos</t>
+          <t>verlassen</t>
         </is>
       </c>
     </row>
@@ -520,7 +520,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>egkataleleimmenos</t>
+          <t>verlassennee</t>
         </is>
       </c>
     </row>
@@ -532,7 +532,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>egkataleleimmenous</t>
+          <t>Verlassenheit</t>
         </is>
       </c>
     </row>
@@ -544,7 +544,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>paraitoumai</t>
+          <t>aufgeben</t>
         </is>
       </c>
     </row>
@@ -556,7 +556,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>paraitoumai</t>
+          <t>aufgeben</t>
         </is>
       </c>
     </row>
@@ -568,7 +568,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>egkataleipo</t>
+          <t>aufgeben</t>
         </is>
       </c>
     </row>
@@ -580,7 +580,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>mone</t>
+          <t>Abtei</t>
         </is>
       </c>
     </row>
@@ -592,7 +592,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>embrontetos</t>
+          <t>betaubt</t>
         </is>
       </c>
     </row>
@@ -604,7 +604,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>zalisma</t>
+          <t>betauben</t>
         </is>
       </c>
     </row>
@@ -616,7 +616,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>amekhania</t>
+          <t>Verwirrung</t>
         </is>
       </c>
     </row>
@@ -628,7 +628,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>ampazour</t>
+          <t>Lampenschirm</t>
         </is>
       </c>
     </row>
@@ -640,7 +640,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>sphageia</t>
+          <t>Schlachthofe</t>
         </is>
       </c>
     </row>
@@ -652,7 +652,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>sphage</t>
+          <t>schlachten</t>
         </is>
       </c>
     </row>
@@ -664,7 +664,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>katarripton</t>
+          <t>Kerl</t>
         </is>
       </c>
     </row>
@@ -676,7 +676,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>sphageio</t>
+          <t>Schlachthof</t>
         </is>
       </c>
     </row>
@@ -688,7 +688,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>katarripto</t>
+          <t>fallen</t>
         </is>
       </c>
     </row>
@@ -700,7 +700,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>khtupemenos</t>
+          <t>niedergeschlagen</t>
         </is>
       </c>
     </row>
@@ -712,7 +712,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>sphaxane</t>
+          <t>geschlachtet</t>
         </is>
       </c>
     </row>
@@ -724,7 +724,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>mone</t>
+          <t>Abtei</t>
         </is>
       </c>
     </row>
@@ -736,7 +736,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>mone</t>
+          <t>Abtei</t>
         </is>
       </c>
     </row>
@@ -748,7 +748,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>abbas</t>
+          <t>abbe</t>
         </is>
       </c>
     </row>
@@ -760,7 +760,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>egoumene</t>
+          <t>Abtissin</t>
         </is>
       </c>
     </row>
@@ -772,7 +772,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>alphabeto</t>
+          <t>ABC</t>
         </is>
       </c>
     </row>
@@ -796,7 +796,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>apostema</t>
+          <t>Abszess</t>
         </is>
       </c>
     </row>
@@ -820,7 +820,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>paraitese</t>
+          <t>Abdankung</t>
         </is>
       </c>
     </row>
@@ -832,7 +832,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>paraitoumai</t>
+          <t>abdanken</t>
         </is>
       </c>
     </row>
@@ -844,7 +844,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>koilia</t>
+          <t>Abdomen</t>
         </is>
       </c>
     </row>
@@ -856,7 +856,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>koiliakos</t>
+          <t>Bauch</t>
         </is>
       </c>
     </row>
@@ -868,7 +868,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>abecedaire</t>
+          <t>Abecedaire</t>
         </is>
       </c>
     </row>
@@ -880,7 +880,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>melissa</t>
+          <t>Biene</t>
         </is>
       </c>
     </row>
@@ -892,7 +892,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>alla</t>
+          <t>aber</t>
         </is>
       </c>
     </row>
@@ -904,7 +904,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>anomalos</t>
+          <t>abweichend</t>
         </is>
       </c>
     </row>
@@ -916,7 +916,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>ektrope</t>
+          <t>Abweichung</t>
         </is>
       </c>
     </row>
@@ -940,7 +940,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>misetes</t>
+          <t>Abscheulicher</t>
         </is>
       </c>
     </row>
@@ -952,7 +952,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Ampitzan</t>
+          <t>Abidjan</t>
         </is>
       </c>
     </row>
@@ -964,7 +964,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>abussos</t>
+          <t>Abgrund</t>
         </is>
       </c>
     </row>
@@ -976,7 +976,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>blabe</t>
+          <t>Schaden</t>
         </is>
       </c>
     </row>
@@ -988,7 +988,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>athlios</t>
+          <t>erbarmlich</t>
         </is>
       </c>
     </row>
@@ -1000,7 +1000,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>athlioteta</t>
+          <t>Verachtung</t>
         </is>
       </c>
     </row>
@@ -1012,7 +1012,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>anakalo dia orkou</t>
+          <t>abschworen</t>
         </is>
       </c>
     </row>
@@ -1024,7 +1024,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>ektome</t>
+          <t>Abtragung</t>
         </is>
       </c>
     </row>
@@ -1036,7 +1036,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>phloios</t>
+          <t>bellen</t>
         </is>
       </c>
     </row>
@@ -1048,7 +1048,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>katargetheke</t>
+          <t>abgeschafft</t>
         </is>
       </c>
     </row>
@@ -1060,7 +1060,7 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>katargo</t>
+          <t>abschaffen</t>
         </is>
       </c>
     </row>
@@ -1072,7 +1072,7 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>katargese</t>
+          <t>Abschaffung</t>
         </is>
       </c>
     </row>
@@ -1084,7 +1084,7 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>katargese</t>
+          <t>Abolitionismus</t>
         </is>
       </c>
     </row>
@@ -1096,7 +1096,7 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>katargetes</t>
+          <t>Abolitionist</t>
         </is>
       </c>
     </row>
@@ -1108,7 +1108,7 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>bdelugma</t>
+          <t>Grauel</t>
         </is>
       </c>
     </row>
@@ -1120,7 +1120,7 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>apekhthes</t>
+          <t>Abscheulichkeit</t>
         </is>
       </c>
     </row>
@@ -1132,7 +1132,7 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>aphthona</t>
+          <t>reichlich</t>
         </is>
       </c>
     </row>
@@ -1144,7 +1144,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>aphthonia</t>
+          <t>Fulle</t>
         </is>
       </c>
     </row>
@@ -1156,7 +1156,7 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>aphthonos</t>
+          <t>reichlich</t>
         </is>
       </c>
     </row>
@@ -1168,7 +1168,7 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>aphthonos</t>
+          <t>reichlich</t>
         </is>
       </c>
     </row>
@@ -1180,7 +1180,7 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>sundrometes</t>
+          <t>Teilnehmer</t>
         </is>
       </c>
     </row>
@@ -1192,7 +1192,7 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>sundrometes</t>
+          <t>Teilnehmer</t>
         </is>
       </c>
     </row>
@@ -1204,7 +1204,7 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>sundrome</t>
+          <t>Abonnement</t>
         </is>
       </c>
     </row>
@@ -1216,7 +1216,7 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>sundromes</t>
+          <t>Abonnements</t>
         </is>
       </c>
     </row>
@@ -1228,7 +1228,7 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>Eggrapheite</t>
+          <t>abonnieren</t>
         </is>
       </c>
     </row>
@@ -1240,7 +1240,7 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>sundromes</t>
+          <t>Abonnements</t>
         </is>
       </c>
     </row>
@@ -1252,7 +1252,7 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>epi tou skaphous</t>
+          <t>an Bord</t>
         </is>
       </c>
     </row>
@@ -1264,7 +1264,7 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>prometheutos</t>
+          <t>erschwinglich</t>
         </is>
       </c>
     </row>
@@ -1276,7 +1276,7 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>sugkrouse</t>
+          <t>Kollision</t>
         </is>
       </c>
     </row>
@@ -1288,7 +1288,7 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>dieuthunseis</t>
+          <t>Adressen</t>
         </is>
       </c>
     </row>
@@ -1300,7 +1300,7 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>dieuthunseis</t>
+          <t>Adressen</t>
         </is>
       </c>
     </row>
@@ -1312,7 +1312,7 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>prosgeionomai</t>
+          <t>landen</t>
         </is>
       </c>
     </row>
@@ -1324,7 +1324,7 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>plesiase</t>
+          <t>naherte sich</t>
         </is>
       </c>
     </row>
@@ -1336,7 +1336,7 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>periballontas KhOROS</t>
+          <t>Umfeld</t>
         </is>
       </c>
     </row>
@@ -1348,7 +1348,7 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>ithagenes</t>
+          <t>Aborigine</t>
         </is>
       </c>
     </row>
@@ -1360,7 +1360,7 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>ithageneis</t>
+          <t>Aborigines</t>
         </is>
       </c>
     </row>
@@ -1372,7 +1372,7 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>anepitukhes</t>
+          <t>fehlgeschlagen</t>
         </is>
       </c>
     </row>
@@ -1384,7 +1384,7 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>skhetika me</t>
+          <t>um</t>
         </is>
       </c>
     </row>
@@ -1396,7 +1396,7 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>epitukhes</t>
+          <t>erfolgreich</t>
         </is>
       </c>
     </row>
@@ -1408,7 +1408,7 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>pherno se peras</t>
+          <t>erreichen</t>
         </is>
       </c>
     </row>
@@ -1420,7 +1420,7 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>tha proekupte</t>
+          <t>wurde ergeben</t>
         </is>
       </c>
     </row>
@@ -1432,7 +1432,7 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>apotelesma</t>
+          <t>Ergebnis</t>
         </is>
       </c>
     </row>
@@ -1444,7 +1444,7 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>apotelesma</t>
+          <t>Ergebnis</t>
         </is>
       </c>
     </row>
@@ -1456,7 +1456,7 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>me apotelesma</t>
+          <t>resultierend</t>
         </is>
       </c>
     </row>
@@ -1468,7 +1468,7 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>na gabgisei</t>
+          <t>Bellen</t>
         </is>
       </c>
     </row>
@@ -1480,7 +1480,7 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>apotribes</t>
+          <t>abrakadabra</t>
         </is>
       </c>
     </row>
@@ -1492,7 +1492,7 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>apoxestiko</t>
+          <t>Schleifmittel</t>
         </is>
       </c>
     </row>
@@ -1504,7 +1504,7 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>tribe</t>
+          <t>Abrieb</t>
         </is>
       </c>
     </row>
@@ -1516,7 +1516,7 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>apoxestiko</t>
+          <t>Schleifmittel</t>
         </is>
       </c>
     </row>
@@ -1528,7 +1528,7 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>sunopsizo</t>
+          <t>abregen</t>
         </is>
       </c>
     </row>
@@ -1540,7 +1540,7 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>abregee</t>
+          <t>abregiert</t>
         </is>
       </c>
     </row>
@@ -1564,7 +1564,7 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>potizo</t>
+          <t>Giessen</t>
         </is>
       </c>
     </row>
@@ -1576,7 +1576,7 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>suntomographia</t>
+          <t>Abkurzung</t>
         </is>
       </c>
     </row>
@@ -1588,7 +1588,7 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>suntomographies</t>
+          <t>Abkurzungen</t>
         </is>
       </c>
     </row>
@@ -1600,7 +1600,7 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>kataphugio</t>
+          <t>Unterschlupf</t>
         </is>
       </c>
     </row>
@@ -1612,7 +1612,7 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>berukokko</t>
+          <t>Aprikose</t>
         </is>
       </c>
     </row>

</xml_diff>